<commit_message>
richard: add extra missing expected var to one negative test case
</commit_message>
<xml_diff>
--- a/rules/CORE-000334/negative/01/data/unit-test-coreid-CG0016-negative.xlsx
+++ b/rules/CORE-000334/negative/01/data/unit-test-coreid-CG0016-negative.xlsx
@@ -482,10 +482,10 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Adverse Events</v>
       </c>
     </row>
@@ -498,7 +498,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -541,35 +541,55 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2" t="str">
+        <v>ta.xpt</v>
+      </c>
+      <c r="C3" s="2" t="str">
+        <v>Dataset</v>
+      </c>
+      <c r="D3" s="2" t="str">
+        <v>N/A</v>
+      </c>
+      <c r="E3" s="2" t="str">
+        <v>$missing_expected_variables</v>
+      </c>
+      <c r="F3" s="2" t="str">
+        <v>TABRANCH</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B4" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C3" s="4" t="str">
+      <c r="C4" s="4" t="str">
         <v>Dataset</v>
       </c>
-      <c r="D3" s="4" t="str">
+      <c r="D4" s="4" t="str">
         <v>N/A</v>
       </c>
-      <c r="E3" s="4" t="str">
+      <c r="E4" s="4" t="str">
         <v>$missing_expected_variables</v>
       </c>
-      <c r="F3" s="4" t="str">
+      <c r="F4" s="4" t="str">
         <v>AEREL</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:H10"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="str">
@@ -594,9 +614,6 @@
         <v>ELEMENT</v>
       </c>
       <c r="H1" s="3" t="str">
-        <v>TABRANCH</v>
-      </c>
-      <c r="I1" s="3" t="str">
         <v>EPOCH</v>
       </c>
     </row>
@@ -623,9 +640,6 @@
         <v>Description of Element</v>
       </c>
       <c r="H2" s="5" t="str">
-        <v>Branch</v>
-      </c>
-      <c r="I2" s="5" t="str">
         <v>Epoch</v>
       </c>
     </row>
@@ -652,9 +666,6 @@
         <v>Char</v>
       </c>
       <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
         <v>Char</v>
       </c>
     </row>
@@ -681,9 +692,6 @@
         <v>13</v>
       </c>
       <c r="H4" s="5">
-        <v>1</v>
-      </c>
-      <c r="I4" s="5">
         <v>9</v>
       </c>
     </row>
@@ -710,9 +718,6 @@
         <v>SCREENING</v>
       </c>
       <c r="H5" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I5" s="4" t="str">
         <v>SCREENING</v>
       </c>
     </row>
@@ -739,9 +744,6 @@
         <v>HUMAN INSULIN</v>
       </c>
       <c r="H6" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I6" s="4" t="str">
         <v>TREATMENT</v>
       </c>
     </row>
@@ -768,9 +770,6 @@
         <v>FOLLOW-UP</v>
       </c>
       <c r="H7" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I7" s="4" t="str">
         <v>FOLLOW-UP</v>
       </c>
     </row>
@@ -797,9 +796,6 @@
         <v>SCREENING</v>
       </c>
       <c r="H8" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I8" s="4" t="str">
         <v>SCREENING</v>
       </c>
     </row>
@@ -826,9 +822,6 @@
         <v>METFORMIN</v>
       </c>
       <c r="H9" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I9" s="4" t="str">
         <v>TREATMENT</v>
       </c>
     </row>
@@ -855,15 +848,12 @@
         <v>FOLLOW-UP</v>
       </c>
       <c r="H10" s="4" t="str">
-        <v/>
-      </c>
-      <c r="I10" s="4" t="str">
         <v>FOLLOW-UP</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H10"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>